<commit_message>
update AI Audit Log
</commit_message>
<xml_diff>
--- a/AI_AuditLog_Example_HoangNhatKha.xlsx
+++ b/AI_AuditLog_Example_HoangNhatKha.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT_UNIVERSITY\Kì 5\5.SWP391\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT_UNIVERSITY\Kì 5\5.SWP391\swp391-aiauditlog-nhatkhaiphone-ux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE0A72FC-B1DF-4AC8-8670-B3410A4BEFBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87411A24-CA6C-490A-BD99-9E08933A8A72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="242">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -628,6 +628,141 @@
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>The SRS needs clearer Introduction, Scope, and Existing Systems sections for the RentalRoom topic.</t>
+  </si>
+  <si>
+    <t>Create Introduction, Scope, and Existing Systems for a RentalRoom search and booking system. Keep it formal for SRS.</t>
+  </si>
+  <si>
+    <t>AI suggested describing RentalRoom as a platform for tenants, landlords, and admin, including searching rooms, posting rooms, booking, deposit, chat, notification, and management.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI provided a good structure but the first version was too general and used broad accommodation examples. Contextualization: Our project is specifically RentalRoom, not hotel booking. Creative Synthesis: I rewrote the content to focus on long-term room rental for students and workers. Decision Ownership: I chose to add these sections before Product Overview to make the SRS more complete and easier to present.</t>
+  </si>
+  <si>
+    <t>Updated SRS Introduction/Scope/Existing Systems section</t>
+  </si>
+  <si>
+    <t>The ERD relationships need to be explained clearly when the teacher asks about one-to-many or many-to-many relations.</t>
+  </si>
+  <si>
+    <t>Explain RentalRoom database relationships such as User-Profile, Room-Booking, Room-Contract, Contract-Payment, and Contract-Occupant in simple terms.</t>
+  </si>
+  <si>
+    <t>AI explained common relationships: one user has one profile, one landlord has many rooms, one room has many booking requests, one rental contract can include multiple occupants, and payments belong to rental contracts.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: The explanation was useful but some relationships needed adjustment to match the actual ERD. Contextualization: In our design, payment and contract logic must follow the deposit/rental flow. Creative Synthesis: I prepared a simplified explanation using examples that can be spoken in presentation. Decision Ownership: I kept only relationships that exist in our database to avoid explaining fake tables.</t>
+  </si>
+  <si>
+    <t>ERD relationship explanation notes</t>
+  </si>
+  <si>
+    <t>The use case diagram may become too complicated if every feature includes Login or Notification.</t>
+  </si>
+  <si>
+    <t>Check whether Login and Send Notification should be included or extended in every RentalRoom use case diagram.</t>
+  </si>
+  <si>
+    <t>AI explained that Login is normally a precondition for protected features, while Notification can be modeled as an included or supporting function only for flows that actually trigger messages.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI was correct, but it may confuse the diagram if overused. Contextualization: The teacher prefers a clean and logical use case diagram. Creative Synthesis: I separated Authentication and used preconditions for login-required functions; notifications are connected only to important events such as booking approval, payment, and cancellation. Decision Ownership: I chose clarity over showing every technical dependency.</t>
+  </si>
+  <si>
+    <t>Use case diagram revision + presentation explanation</t>
+  </si>
+  <si>
+    <t>The room booking process needs a clear status lifecycle from request to deposit to rental contract.</t>
+  </si>
+  <si>
+    <t>Design a status flow for rental request and room reservation in RentalRoom after tenant views a room and wants to rent it.</t>
+  </si>
+  <si>
+    <t>AI suggested statuses such as Pending, Approved, Pending Payment, Deposited, Contract Created, Rejected, Cancelled, and Expired.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI's status list is helpful but needs rules for who can change each status. Contextualization: Landlord approves the request first, then tenant pays deposit before the contract is created. Creative Synthesis: I created a lifecycle: Request Submitted → Approved → Pending Deposit → Deposited → Contract Created; failure paths include Rejected, Cancelled, and Expired. Decision Ownership: This flow was selected because it matches the team's business rule: view room, deposit, then rent room.</t>
+  </si>
+  <si>
+    <t>State diagram / booking flow update</t>
+  </si>
+  <si>
+    <t>The team needs weekly Jira update content showing what was completed for the SRS and AI audit log.</t>
+  </si>
+  <si>
+    <t>Write a short Jira week update for completing RentalRoom SRS Introduction, Scope, Existing Systems, and AI Audit Log entries.</t>
+  </si>
+  <si>
+    <t>AI suggested a concise update: completed SRS sections, updated audit log entries, reviewed hallucination cases, and prepared evidence for presentation.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI output was acceptable but too generic. Contextualization: The update must match the actual tasks completed this week. Creative Synthesis: I customized the update to mention RentalRoom SRS, database/use case explanation, booking status flow, and audit log update. Decision Ownership: I used this wording so the Jira record is specific and traceable.</t>
+  </si>
+  <si>
+    <t>Jira Week 2 update/comment</t>
+  </si>
+  <si>
+    <t>Existing systems for RentalRoom can be described mainly using hotel booking platforms.</t>
+  </si>
+  <si>
+    <t>Rental request only needs Approved and Rejected statuses.</t>
+  </si>
+  <si>
+    <t>Hotel booking platforms are related but not fully the same as long-term room rental systems for students/workers.</t>
+  </si>
+  <si>
+    <t>The booking flow also needs Pending Deposit, Deposited, Cancelled, and Expired to handle real business cases.</t>
+  </si>
+  <si>
+    <t>Compared the topic name and scope with RentalRoom business requirements.</t>
+  </si>
+  <si>
+    <t>Checked the flow from viewing room → landlord approval → deposit → rental contract.</t>
+  </si>
+  <si>
+    <t>Rewrote Existing Systems to include Facebook Marketplace, Chợ Tốt, Phongtro123, Airbnb/Booking only as comparable references.</t>
+  </si>
+  <si>
+    <t>Added a clearer status lifecycle for rental request and payment deadline.</t>
+  </si>
+  <si>
+    <t>Có – chọn filter truyền thống làm core vì dễ test và đúng yêu cầu tìm phòng</t>
+  </si>
+  <si>
+    <t>Có – thêm RentalContract/Occupant để quản lý lịch sử thuê và nhiều người ở chung</t>
+  </si>
+  <si>
+    <t>Có – phát hiện currentTenantId trong Room không đủ cho lịch sử thuê</t>
+  </si>
+  <si>
+    <t>Có – thêm deadline thanh toán để tránh landlord phải chờ quá lâu</t>
+  </si>
+  <si>
+    <t>Có – Login nên là precondition để use case diagram gọn hơn</t>
+  </si>
+  <si>
+    <t>Có – Scope/Existing Systems giúp SRS đúng chủ đề RentalRoom</t>
+  </si>
+  <si>
+    <t>Có – thêm transactionId để tránh lỗi payment trùng hoặc sai trạng thái</t>
+  </si>
+  <si>
+    <t>Có – Introduction/Scope cần tập trung vào thuê phòng dài hạn</t>
+  </si>
+  <si>
+    <t>Có – giải thích quan hệ ERD bằng ví dụ để dễ trình bày với giáo viên</t>
+  </si>
+  <si>
+    <t>Có – tách Authentication và Notification để diagram không bị rối</t>
+  </si>
+  <si>
+    <t>Có – status lifecycle giúp booking flow rõ từ request đến contract</t>
+  </si>
+  <si>
+    <t>Có – Jira update cần cụ thể task đã làm trong tuần 2</t>
   </si>
 </sst>
 </file>
@@ -802,7 +937,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -837,22 +972,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -876,6 +995,25 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1190,14 +1328,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
     </row>
     <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -1245,24 +1383,24 @@
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="22">
-        <v>60</v>
+      <c r="C10" s="16">
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="23">
-        <v>10</v>
+      <c r="C11" s="17">
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="24">
-        <v>0.16669999999999999</v>
+      <c r="C12" s="18">
+        <v>0.2</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>10</v>
@@ -1272,8 +1410,8 @@
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="23">
-        <v>3</v>
+      <c r="C13" s="17">
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" x14ac:dyDescent="0.35">
@@ -1299,7 +1437,7 @@
       <c r="A17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="19" t="s">
         <v>106</v>
       </c>
       <c r="C17" s="5" t="s">
@@ -1310,30 +1448,30 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="19" t="s">
         <v>108</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="25" t="s">
+      <c r="D18" s="19" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="C19" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="25" t="s">
+      <c r="D19" s="19" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1341,27 +1479,27 @@
       <c r="A20" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="C20" s="25" t="s">
+      <c r="C20" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D20" s="25" t="s">
+      <c r="D20" s="19" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D21" s="22" t="s">
+      <c r="D21" s="16" t="s">
         <v>119</v>
       </c>
     </row>
@@ -1397,7 +1535,7 @@
         <v>27</v>
       </c>
       <c r="B25" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>26</v>
@@ -1419,7 +1557,7 @@
         <v>29</v>
       </c>
       <c r="B27" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>26</v>
@@ -1448,28 +1586,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
     </row>
     <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
@@ -1507,19 +1645,19 @@
       <c r="C4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="19" t="s">
         <v>150</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="E4" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="25" t="s">
+      <c r="F4" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="G4" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="19" t="s">
         <v>122</v>
       </c>
     </row>
@@ -1527,25 +1665,25 @@
       <c r="A5" s="5">
         <v>2</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="F5" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="H5" s="25" t="s">
+      <c r="H5" s="19" t="s">
         <v>125</v>
       </c>
     </row>
@@ -1553,25 +1691,25 @@
       <c r="A6" s="5">
         <v>3</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="F6" s="25" t="s">
+      <c r="F6" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="H6" s="25" t="s">
+      <c r="H6" s="19" t="s">
         <v>128</v>
       </c>
     </row>
@@ -1579,25 +1717,25 @@
       <c r="A7" s="5">
         <v>4</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="F7" s="25" t="s">
+      <c r="F7" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="G7" s="25" t="s">
+      <c r="G7" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="H7" s="25" t="s">
+      <c r="H7" s="19" t="s">
         <v>131</v>
       </c>
     </row>
@@ -1605,25 +1743,25 @@
       <c r="A8" s="5">
         <v>5</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F8" s="25" t="s">
+      <c r="F8" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G8" s="25" t="s">
+      <c r="G8" s="19" t="s">
         <v>164</v>
       </c>
-      <c r="H8" s="25" t="s">
+      <c r="H8" s="19" t="s">
         <v>136</v>
       </c>
     </row>
@@ -1631,25 +1769,25 @@
       <c r="A9" s="5">
         <v>6</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="D9" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="F9" s="25" t="s">
+      <c r="F9" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="G9" s="25" t="s">
+      <c r="G9" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="H9" s="25" t="s">
+      <c r="H9" s="19" t="s">
         <v>137</v>
       </c>
     </row>
@@ -1657,25 +1795,25 @@
       <c r="A10" s="5">
         <v>7</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="19" t="s">
         <v>156</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="F10" s="25" t="s">
+      <c r="F10" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="G10" s="25" t="s">
+      <c r="G10" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="H10" s="25" t="s">
+      <c r="H10" s="19" t="s">
         <v>140</v>
       </c>
     </row>
@@ -1683,25 +1821,25 @@
       <c r="A11" s="5">
         <v>8</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="F11" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="G11" s="25" t="s">
+      <c r="G11" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="H11" s="25" t="s">
+      <c r="H11" s="19" t="s">
         <v>143</v>
       </c>
     </row>
@@ -1709,25 +1847,25 @@
       <c r="A12" s="5">
         <v>9</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="F12" s="25" t="s">
+      <c r="F12" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="G12" s="25" t="s">
+      <c r="G12" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="H12" s="25" t="s">
+      <c r="H12" s="19" t="s">
         <v>146</v>
       </c>
     </row>
@@ -1735,77 +1873,157 @@
       <c r="A13" s="5">
         <v>10</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="E13" s="25" t="s">
+      <c r="E13" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="F13" s="25" t="s">
+      <c r="F13" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="G13" s="25" t="s">
+      <c r="G13" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="H13" s="25" t="s">
+      <c r="H13" s="19" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-    </row>
-    <row r="15" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-    </row>
-    <row r="16" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-    </row>
-    <row r="17" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-    </row>
-    <row r="18" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
+    <row r="14" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="19">
+        <v>11</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>199</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="H14" s="19" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="5">
+        <v>12</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>202</v>
+      </c>
+      <c r="E15" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="F15" s="19" t="s">
+        <v>204</v>
+      </c>
+      <c r="G15" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="H15" s="19" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="5">
+        <v>13</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="H16" s="19" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="5">
+        <v>14</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="E17" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="H17" s="19" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="5">
+        <v>15</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>220</v>
+      </c>
+      <c r="H18" s="19" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
@@ -1907,24 +2125,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
     </row>
     <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
@@ -1950,19 +2168,19 @@
       <c r="A4" s="5">
         <v>2</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="E4" s="19" t="s">
         <v>172</v>
       </c>
-      <c r="F4" s="25" t="s">
+      <c r="F4" s="19" t="s">
         <v>173</v>
       </c>
     </row>
@@ -1970,19 +2188,19 @@
       <c r="A5" s="5">
         <v>6</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="19" t="s">
         <v>178</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="19" t="s">
         <v>175</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="F5" s="19" t="s">
         <v>176</v>
       </c>
     </row>
@@ -1990,37 +2208,61 @@
       <c r="A6" s="5">
         <v>10</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="F6" s="25" t="s">
+      <c r="F6" s="19" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-    </row>
-    <row r="8" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
+    <row r="7" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>11</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>222</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>14</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>223</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="9" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
@@ -2232,7 +2474,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2242,20 +2484,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -2283,10 +2525,10 @@
       <c r="B6" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C6" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="22" t="s">
         <v>183</v>
       </c>
     </row>
@@ -2297,10 +2539,10 @@
       <c r="B7" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="22" t="s">
         <v>184</v>
       </c>
     </row>
@@ -2311,10 +2553,10 @@
       <c r="B8" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="D8" s="22" t="s">
         <v>185</v>
       </c>
     </row>
@@ -2325,10 +2567,10 @@
       <c r="B9" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="D9" s="23" t="s">
         <v>186</v>
       </c>
     </row>
@@ -2339,10 +2581,10 @@
       <c r="B10" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="D10" s="28" t="s">
+      <c r="D10" s="22" t="s">
         <v>187</v>
       </c>
     </row>
@@ -2372,10 +2614,10 @@
       <c r="B14" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="D14" s="28" t="s">
+      <c r="D14" s="22" t="s">
         <v>188</v>
       </c>
     </row>
@@ -2386,10 +2628,10 @@
       <c r="B15" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="D15" s="28" t="s">
+      <c r="D15" s="22" t="s">
         <v>189</v>
       </c>
     </row>
@@ -2400,10 +2642,10 @@
       <c r="B16" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="D16" s="28" t="s">
+      <c r="D16" s="22" t="s">
         <v>190</v>
       </c>
     </row>
@@ -2414,10 +2656,10 @@
       <c r="B17" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="22" t="s">
         <v>191</v>
       </c>
     </row>
@@ -2428,10 +2670,10 @@
       <c r="B18" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="22" t="s">
         <v>192</v>
       </c>
     </row>
@@ -2513,6 +2755,174 @@
         <v>196</v>
       </c>
       <c r="D30" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="30">
+        <v>4</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>230</v>
+      </c>
+      <c r="C31" t="s">
+        <v>196</v>
+      </c>
+      <c r="D31" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="30">
+        <v>5</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>231</v>
+      </c>
+      <c r="C32" t="s">
+        <v>196</v>
+      </c>
+      <c r="D32" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="30">
+        <v>6</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>232</v>
+      </c>
+      <c r="C33" t="s">
+        <v>196</v>
+      </c>
+      <c r="D33" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="30">
+        <v>7</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="C34" t="s">
+        <v>196</v>
+      </c>
+      <c r="D34" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="30">
+        <v>8</v>
+      </c>
+      <c r="B35" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="C35" t="s">
+        <v>196</v>
+      </c>
+      <c r="D35" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="30">
+        <v>9</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="C36" t="s">
+        <v>196</v>
+      </c>
+      <c r="D36" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="30">
+        <v>10</v>
+      </c>
+      <c r="B37" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="C37" t="s">
+        <v>196</v>
+      </c>
+      <c r="D37" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="30">
+        <v>11</v>
+      </c>
+      <c r="B38" s="16" t="s">
+        <v>237</v>
+      </c>
+      <c r="C38" t="s">
+        <v>196</v>
+      </c>
+      <c r="D38" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="30">
+        <v>12</v>
+      </c>
+      <c r="B39" s="16" t="s">
+        <v>238</v>
+      </c>
+      <c r="C39" t="s">
+        <v>196</v>
+      </c>
+      <c r="D39" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="30">
+        <v>13</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>239</v>
+      </c>
+      <c r="C40" t="s">
+        <v>196</v>
+      </c>
+      <c r="D40" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="30">
+        <v>14</v>
+      </c>
+      <c r="B41" s="16" t="s">
+        <v>240</v>
+      </c>
+      <c r="C41" t="s">
+        <v>196</v>
+      </c>
+      <c r="D41" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="30">
+        <v>15</v>
+      </c>
+      <c r="B42" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="C42" t="s">
+        <v>196</v>
+      </c>
+      <c r="D42" t="s">
         <v>196</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update:week 3 and week 4 AI AuditLog
</commit_message>
<xml_diff>
--- a/AI_AuditLog_Example_HoangNhatKha.xlsx
+++ b/AI_AuditLog_Example_HoangNhatKha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT_UNIVERSITY\Kì 5\5.SWP391\swp391-aiauditlog-nhatkhaiphone-ux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87411A24-CA6C-490A-BD99-9E08933A8A72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11BBBB51-C21D-44FF-8BE5-9EDB05E1625C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="314">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -763,6 +763,222 @@
   </si>
   <si>
     <t>Có – Jira update cần cụ thể task đã làm trong tuần 2</t>
+  </si>
+  <si>
+    <t>Week 3 starts frontend implementation, so the UI must be broken into clear pages and reusable components.</t>
+  </si>
+  <si>
+    <t>Break down the RentalRoom frontend into pages, components, and user flows for Tenant, Landlord, and Admin.</t>
+  </si>
+  <si>
+    <t>AI suggested pages: Home, Room List, Room Detail, Login/Register, Tenant Dashboard, Landlord Room Management, Booking/Request, Profile, and Admin moderation.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI gave a good structure, but I reduced it to screens needed for the current sprint. Contextualization: focus on Tenant search flow and auth screens first. Verification: compared with use case diagram. Decision: create reusable components such as Navbar, RoomCard, FilterBar, AuthForm, and ProfileForm.</t>
+  </si>
+  <si>
+    <t>Frontend sitemap + component folder draft</t>
+  </si>
+  <si>
+    <t>The room search UI needs to support common user behavior: search by location, filter by price, and view room details.</t>
+  </si>
+  <si>
+    <t>Design the frontend flow for searching rental rooms with filters and room cards.</t>
+  </si>
+  <si>
+    <t>AI suggested a search bar, filter panel, room cards with price/location/area, and a detail page with images and contact/request buttons.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: The suggestion fits user behavior, but some fields were too complex for week 3. Contextualization: keep location, price range, room type, and facilities. Verification: matched with RentalRoom search use case. Decision: separate SearchPage, FilterSidebar, RoomList, and RoomCard components.</t>
+  </si>
+  <si>
+    <t>Search page wireframe + component list</t>
+  </si>
+  <si>
+    <t>The UI design needs consistent layout and naming so that the team can code React components without confusion.</t>
+  </si>
+  <si>
+    <t>Suggest a clean React frontend structure and naming convention for a rental room web app.</t>
+  </si>
+  <si>
+    <t>AI suggested organizing src into components, pages, services, hooks, assets, and routes, with PascalCase component names.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI structure is useful but too broad for a small student project. Contextualization: keep components/pages/routes/services only. Verification: checked against current React project structure. Decision: use simple folders to avoid overengineering.</t>
+  </si>
+  <si>
+    <t>React folder structure screenshot</t>
+  </si>
+  <si>
+    <t>The AI suggested only desktop UI, but the system will likely be used on phones by tenants.</t>
+  </si>
+  <si>
+    <t>Check possible issues in a desktop-first RentalRoom frontend design.</t>
+  </si>
+  <si>
+    <t>AI identified risks such as small filter sidebar on mobile, overcrowded room cards, and difficult form input on small screens.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: HALLUCINATION/OVERSIMPLIFICATION DETECTED: the first UI plan ignored responsive behavior. Contextualization: most tenants may search using mobile. Verification: reviewed screen widths in browser dev tools. Decision: make filter collapsible on mobile and room cards stack vertically.</t>
+  </si>
+  <si>
+    <t>Responsive UI checklist</t>
+  </si>
+  <si>
+    <t>The Login/Register/Forgot Password pages need validation rules before connecting to backend.</t>
+  </si>
+  <si>
+    <t>Write frontend validation rules for login, register, forgot password, and update profile forms.</t>
+  </si>
+  <si>
+    <t>AI suggested required email/password, password length, confirm password matching, phone format, and avatar/file validation.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI's rules are mostly correct, but password policy should not be too strict for prototype. Contextualization: apply basic validation first. Verification: tested invalid input cases manually. Decision: show inline error messages and disable submit when required fields are invalid.</t>
+  </si>
+  <si>
+    <t>Auth form validation notes</t>
+  </si>
+  <si>
+    <t>Week 4 starts backend authentication, so the backend auth module must be separated into API endpoints and services.</t>
+  </si>
+  <si>
+    <t>Break down backend authentication features for RentalRoom: register, login, logout, Google login, forgot password, update profile.</t>
+  </si>
+  <si>
+    <t>AI suggested controllers/services/routes for Auth, User/Profile, OTP/Email, Google OAuth, and token handling.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI decomposition is suitable, but Google login and OTP require external services. Contextualization: implement normal auth first, then Google/forgot password. Verification: compared with sprint scope. Decision: separate auth.controller, auth.service, profile.controller, and middleware/authMiddleware.</t>
+  </si>
+  <si>
+    <t>Backend auth module plan</t>
+  </si>
+  <si>
+    <t>The database needs fields and relationships to support authentication and user profile updates.</t>
+  </si>
+  <si>
+    <t>Design database fields for users, profiles, OTP reset, and Google login in RentalRoom.</t>
+  </si>
+  <si>
+    <t>AI suggested Users table with email, passwordHash, role, status, googleId, createdAt; Profiles table with fullName, phone, avatar, address; PasswordResetOtp table.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI output is good but must not store raw password or raw OTP. Contextualization: store passwordHash and hashed OTP/expiry. Verification: checked security requirements. Decision: update schema with passwordHash, provider, googleId, resetOtpHash, resetOtpExpires.</t>
+  </si>
+  <si>
+    <t>Auth database schema update</t>
+  </si>
+  <si>
+    <t>The AI recommended storing JWT in localStorage, but this may create security issues.</t>
+  </si>
+  <si>
+    <t>Verify whether JWT should be stored in localStorage or httpOnly cookie for a rental room web app.</t>
+  </si>
+  <si>
+    <t>AI explained localStorage is easier but vulnerable to XSS, while httpOnly cookies reduce token theft risk.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: HALLUCINATION/OVERSIMPLIFICATION DETECTED: the first recommendation was too simple for authentication security. Contextualization: use httpOnly cookie or safer token handling for backend auth. Verification: discussed XSS risk and logout behavior. Decision: avoid relying only on localStorage for sensitive token storage.</t>
+  </si>
+  <si>
+    <t>Auth security note + token handling decision</t>
+  </si>
+  <si>
+    <t>Forgot password flow must be secure and should not reveal whether an email exists.</t>
+  </si>
+  <si>
+    <t>Write backend flow for forgot password using OTP/email verification.</t>
+  </si>
+  <si>
+    <t>AI suggested request reset → generate OTP → email OTP → verify OTP → set new password → invalidate OTP.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI flow is correct, but the response message should be generic. Contextualization: avoid user enumeration. Verification: checked edge cases: expired OTP, wrong OTP, reused OTP. Decision: return 'If the email exists, an OTP has been sent' and limit OTP attempts.</t>
+  </si>
+  <si>
+    <t>Forgot password API flow</t>
+  </si>
+  <si>
+    <t>Update profile must not allow users to change protected fields such as role or account status.</t>
+  </si>
+  <si>
+    <t>Check security risks when implementing update profile API.</t>
+  </si>
+  <si>
+    <t>AI identified mass assignment risk, missing authentication middleware, and lack of file validation for avatar upload.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI correctly found risks, but implementation must whitelist fields. Contextualization: users can update name, phone, address, avatar only. Verification: reviewed request body fields. Decision: reject role/status changes and require authenticated user for profile update.</t>
+  </si>
+  <si>
+    <t>Update profile validation checklist</t>
+  </si>
+  <si>
+    <t>Desktop UI design is enough for the first frontend sprint.</t>
+  </si>
+  <si>
+    <t>JWT can simply be stored in localStorage for login sessions.</t>
+  </si>
+  <si>
+    <t>Forgot password API can say 'email not found' when the account does not exist.</t>
+  </si>
+  <si>
+    <t>Tenants often search rooms on mobile, so responsive behavior is necessary.</t>
+  </si>
+  <si>
+    <t>localStorage is vulnerable to token theft through XSS; safer handling is needed for authentication.</t>
+  </si>
+  <si>
+    <t>This can reveal registered emails and create user enumeration risk.</t>
+  </si>
+  <si>
+    <t>Reviewed frontend screen in browser dev tools and checked search/filter usability on smaller width.</t>
+  </si>
+  <si>
+    <t>Compared token storage risks and reviewed logout/session behavior.</t>
+  </si>
+  <si>
+    <t>Checked security edge cases for forgot password flow.</t>
+  </si>
+  <si>
+    <t>Added responsive rules: collapsible filter, stacked room cards, and mobile-friendly form spacing.</t>
+  </si>
+  <si>
+    <t>Avoid relying only on localStorage; prefer httpOnly cookie or safer token strategy.</t>
+  </si>
+  <si>
+    <t>Use generic response: 'If the email exists, an OTP has been sent', and limit OTP attempts.</t>
+  </si>
+  <si>
+    <t>Có – tách frontend thành page/component để team dễ chia việc và code React</t>
+  </si>
+  <si>
+    <t>Có – search/filter UI bám sát hành vi tenant tìm phòng</t>
+  </si>
+  <si>
+    <t>Có – folder structure đơn giản giúp tránh overengineering</t>
+  </si>
+  <si>
+    <t>Có – phát hiện UI desktop-first thiếu responsive mobile</t>
+  </si>
+  <si>
+    <t>Có – validation frontend giúp giảm lỗi trước khi gọi API</t>
+  </si>
+  <si>
+    <t>Có – tách auth backend thành controller/service/middleware rõ ràng</t>
+  </si>
+  <si>
+    <t>Có – schema auth cần passwordHash, Google ID và OTP reset an toàn</t>
+  </si>
+  <si>
+    <t>Có – token storage cần cân nhắc bảo mật thay vì chỉ localStorage</t>
+  </si>
+  <si>
+    <t>Có – forgot password phải tránh lộ email tồn tại trong hệ thống</t>
+  </si>
+  <si>
+    <t>Có – update profile phải whitelist field để tránh đổi role/status</t>
   </si>
 </sst>
 </file>
@@ -937,7 +1153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -996,6 +1212,9 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1012,8 +1231,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1328,14 +1553,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
     </row>
     <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -1384,7 +1609,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="16">
-        <v>70</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1392,7 +1617,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="17">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1400,7 +1625,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="18">
-        <v>0.2</v>
+        <v>0.17860000000000001</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>10</v>
@@ -1411,7 +1636,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="17">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" x14ac:dyDescent="0.35">
@@ -1524,7 +1749,7 @@
         <v>25</v>
       </c>
       <c r="B24" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>26</v>
@@ -1535,7 +1760,7 @@
         <v>27</v>
       </c>
       <c r="B25" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>26</v>
@@ -1546,7 +1771,7 @@
         <v>28</v>
       </c>
       <c r="B26" s="6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>26</v>
@@ -1557,7 +1782,7 @@
         <v>29</v>
       </c>
       <c r="B27" s="6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>26</v>
@@ -1573,7 +1798,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1586,28 +1811,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
@@ -2025,85 +2250,265 @@
         <v>221</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-    </row>
-    <row r="20" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="21" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-    </row>
-    <row r="22" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-    </row>
-    <row r="23" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-    </row>
-    <row r="24" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-    </row>
-    <row r="25" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-    </row>
-    <row r="26" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
+    <row r="19" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="19">
+        <v>16</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>242</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="H19" s="19" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="19">
+        <v>17</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="F20" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="G20" s="19" t="s">
+        <v>250</v>
+      </c>
+      <c r="H20" s="19" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="19">
+        <v>18</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>252</v>
+      </c>
+      <c r="E21" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>254</v>
+      </c>
+      <c r="G21" s="19" t="s">
+        <v>255</v>
+      </c>
+      <c r="H21" s="19" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="19">
+        <v>19</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>257</v>
+      </c>
+      <c r="E22" s="19" t="s">
+        <v>258</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>259</v>
+      </c>
+      <c r="G22" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="H22" s="19" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="19">
+        <v>20</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>262</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>263</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>264</v>
+      </c>
+      <c r="G23" s="19" t="s">
+        <v>265</v>
+      </c>
+      <c r="H23" s="19" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="19">
+        <v>21</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>267</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>268</v>
+      </c>
+      <c r="F24" s="19" t="s">
+        <v>269</v>
+      </c>
+      <c r="G24" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="H24" s="19" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="19">
+        <v>22</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>272</v>
+      </c>
+      <c r="E25" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="F25" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="G25" s="19" t="s">
+        <v>275</v>
+      </c>
+      <c r="H25" s="19" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="123.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="19">
+        <v>23</v>
+      </c>
+      <c r="B26" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" s="19" t="s">
+        <v>277</v>
+      </c>
+      <c r="E26" s="19" t="s">
+        <v>278</v>
+      </c>
+      <c r="F26" s="19" t="s">
+        <v>279</v>
+      </c>
+      <c r="G26" s="19" t="s">
+        <v>280</v>
+      </c>
+      <c r="H26" s="19" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="31">
+        <v>24</v>
+      </c>
+      <c r="B27" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="31" t="s">
+        <v>29</v>
+      </c>
+      <c r="D27" s="31" t="s">
+        <v>282</v>
+      </c>
+      <c r="E27" s="31" t="s">
+        <v>283</v>
+      </c>
+      <c r="F27" s="31" t="s">
+        <v>284</v>
+      </c>
+      <c r="G27" s="31" t="s">
+        <v>285</v>
+      </c>
+      <c r="H27" s="31" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="66" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="31">
+        <v>25</v>
+      </c>
+      <c r="B28" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" s="31" t="s">
+        <v>287</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>288</v>
+      </c>
+      <c r="F28" s="31" t="s">
+        <v>289</v>
+      </c>
+      <c r="G28" s="31" t="s">
+        <v>290</v>
+      </c>
+      <c r="H28" s="31" t="s">
+        <v>291</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2125,24 +2530,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
@@ -2264,29 +2669,65 @@
         <v>229</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-    </row>
-    <row r="10" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-    </row>
-    <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
+    <row r="9" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="19">
+        <v>19</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>292</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>295</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="19">
+        <v>23</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>293</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>296</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="19">
+        <v>24</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>294</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>303</v>
+      </c>
     </row>
     <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
@@ -2474,7 +2915,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2484,20 +2925,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -2759,7 +3200,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="30">
+      <c r="A31" s="24">
         <v>4</v>
       </c>
       <c r="B31" s="16" t="s">
@@ -2773,7 +3214,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="30">
+      <c r="A32" s="24">
         <v>5</v>
       </c>
       <c r="B32" s="16" t="s">
@@ -2787,7 +3228,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="30">
+      <c r="A33" s="24">
         <v>6</v>
       </c>
       <c r="B33" s="16" t="s">
@@ -2801,7 +3242,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="30">
+      <c r="A34" s="24">
         <v>7</v>
       </c>
       <c r="B34" s="16" t="s">
@@ -2815,7 +3256,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="30">
+      <c r="A35" s="24">
         <v>8</v>
       </c>
       <c r="B35" s="16" t="s">
@@ -2829,7 +3270,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="30">
+      <c r="A36" s="24">
         <v>9</v>
       </c>
       <c r="B36" s="16" t="s">
@@ -2843,7 +3284,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="30">
+      <c r="A37" s="24">
         <v>10</v>
       </c>
       <c r="B37" s="16" t="s">
@@ -2857,7 +3298,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="30">
+      <c r="A38" s="24">
         <v>11</v>
       </c>
       <c r="B38" s="16" t="s">
@@ -2871,7 +3312,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="30">
+      <c r="A39" s="24">
         <v>12</v>
       </c>
       <c r="B39" s="16" t="s">
@@ -2885,7 +3326,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="30">
+      <c r="A40" s="24">
         <v>13</v>
       </c>
       <c r="B40" s="16" t="s">
@@ -2899,7 +3340,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="30">
+      <c r="A41" s="24">
         <v>14</v>
       </c>
       <c r="B41" s="16" t="s">
@@ -2913,7 +3354,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="30">
+      <c r="A42" s="24">
         <v>15</v>
       </c>
       <c r="B42" s="16" t="s">
@@ -2923,6 +3364,146 @@
         <v>196</v>
       </c>
       <c r="D42" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A43" s="32">
+        <v>16</v>
+      </c>
+      <c r="B43" s="31" t="s">
+        <v>304</v>
+      </c>
+      <c r="C43" t="s">
+        <v>196</v>
+      </c>
+      <c r="D43" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="33">
+        <v>17</v>
+      </c>
+      <c r="B44" s="31" t="s">
+        <v>305</v>
+      </c>
+      <c r="C44" t="s">
+        <v>196</v>
+      </c>
+      <c r="D44" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="24">
+        <v>18</v>
+      </c>
+      <c r="B45" s="31" t="s">
+        <v>306</v>
+      </c>
+      <c r="C45" t="s">
+        <v>196</v>
+      </c>
+      <c r="D45" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" s="24">
+        <v>19</v>
+      </c>
+      <c r="B46" s="31" t="s">
+        <v>307</v>
+      </c>
+      <c r="C46" t="s">
+        <v>196</v>
+      </c>
+      <c r="D46" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="24">
+        <v>20</v>
+      </c>
+      <c r="B47" s="31" t="s">
+        <v>308</v>
+      </c>
+      <c r="C47" t="s">
+        <v>196</v>
+      </c>
+      <c r="D47" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="24">
+        <v>21</v>
+      </c>
+      <c r="B48" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="C48" t="s">
+        <v>196</v>
+      </c>
+      <c r="D48" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="24">
+        <v>22</v>
+      </c>
+      <c r="B49" s="31" t="s">
+        <v>310</v>
+      </c>
+      <c r="C49" t="s">
+        <v>196</v>
+      </c>
+      <c r="D49" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="24">
+        <v>23</v>
+      </c>
+      <c r="B50" s="31" t="s">
+        <v>311</v>
+      </c>
+      <c r="C50" t="s">
+        <v>196</v>
+      </c>
+      <c r="D50" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="24">
+        <v>24</v>
+      </c>
+      <c r="B51" s="31" t="s">
+        <v>312</v>
+      </c>
+      <c r="C51" t="s">
+        <v>196</v>
+      </c>
+      <c r="D51" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="24">
+        <v>25</v>
+      </c>
+      <c r="B52" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="C52" t="s">
+        <v>196</v>
+      </c>
+      <c r="D52" t="s">
         <v>196</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update: Week5 AI AuditLog
</commit_message>
<xml_diff>
--- a/AI_AuditLog_Example_HoangNhatKha.xlsx
+++ b/AI_AuditLog_Example_HoangNhatKha.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT_UNIVERSITY\Kì 5\5.SWP391\swp391-aiauditlog-nhatkhaiphone-ux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11BBBB51-C21D-44FF-8BE5-9EDB05E1625C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA812718-B8B6-4D11-8A6D-6E2826D34677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="352">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -979,6 +979,120 @@
   </si>
   <si>
     <t>Có – update profile phải whitelist field để tránh đổi role/status</t>
+  </si>
+  <si>
+    <t>Week 5 starts backend implementation for Landlord features, so the module must be separated into clear APIs and services.</t>
+  </si>
+  <si>
+    <t>Break down backend features for Landlord in RentalRoom: manage rooms, view rental requests, approve/reject requests, manage contracts, and dashboard data.</t>
+  </si>
+  <si>
+    <t>AI suggested separating LandlordRoom, RentalRequest, Contract, ViewingSchedule, PaymentSummary, and Dashboard services/routes.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI decomposition is useful but too broad for one sprint. Contextualization: Week 5 focuses on core Landlord backend only. Verification: compared with use case diagram and current database tables. Decision: implement room CRUD, rental request approval/rejection, contract creation support, and landlord dashboard summary first.</t>
+  </si>
+  <si>
+    <t>Landlord backend API plan</t>
+  </si>
+  <si>
+    <t>Landlord needs APIs to create, update, and delete room posts with images, facilities, price, address, and availability status.</t>
+  </si>
+  <si>
+    <t>Design backend validation rules and API flow for Landlord creating/updating rental room posts.</t>
+  </si>
+  <si>
+    <t>AI suggested validating required fields, price &gt; 0, area &gt; 0, address not empty, image list, facilities list, and room ownership before update/delete.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI rules are correct but image upload can be simplified for prototype. Contextualization: use image URLs or uploaded file paths depending on team implementation. Verification: checked database fields Room, RoomImage, Facility, RoomFacility. Decision: validate core room data first and handle facilities/images through separate related tables.</t>
+  </si>
+  <si>
+    <t>Room CRUD API validation notes</t>
+  </si>
+  <si>
+    <t>Landlord must review tenant rental requests and decide whether to approve or reject them before deposit payment.</t>
+  </si>
+  <si>
+    <t>Write backend flow for Landlord approving or rejecting a rental request in RentalRoom.</t>
+  </si>
+  <si>
+    <t>AI suggested: get pending requests for landlord's rooms → check request status → approve/reject → update status → notify tenant → if approved, set Pending Deposit.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI flow matches the business rule but must prevent approving invalid or already processed requests. Contextualization: landlord approval happens before tenant deposit. Verification: matched with rental request status lifecycle. Decision: allow transition only from Pending to Approved/Pending Deposit or Rejected.</t>
+  </si>
+  <si>
+    <t>Rental request approval API flow</t>
+  </si>
+  <si>
+    <t>Landlord backend APIs have a security risk if they only use roomId/requestId without checking ownership.</t>
+  </si>
+  <si>
+    <t>Check authorization risks for Landlord room and rental request APIs.</t>
+  </si>
+  <si>
+    <t>AI warned that a landlord could update another landlord's room if the API only checks login and not resource ownership.</t>
+  </si>
+  <si>
+    <t>Landlord authorization checklist</t>
+  </si>
+  <si>
+    <t>Critical Thinking: HALLUCINATION/OVERSIMPLIFICATION DETECTED: a simple role check is not enough. Contextualization: each landlord can only manage rooms they created. Verification: reviewed API parameters and database relationship User → Room. Decision: every update/delete/approve/reject query must include landlordId ownership condition.</t>
+  </si>
+  <si>
+    <t>After a tenant pays deposit, the system needs backend logic so landlord can create or confirm a rental contract correctly.</t>
+  </si>
+  <si>
+    <t>Design backend flow connecting approved request, deposit payment, and contract creation for Landlord.</t>
+  </si>
+  <si>
+    <t>AI suggested checking payment success, request status, room availability, tenant information, contract dates, deposit amount, and then creating Contract with status Active/Pending Sign.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI gave a good flow but the contract should not be created from unpaid requests. Contextualization: team rule is view room → deposit → rent room/contract. Verification: compared with Payment and Contract entities. Decision: create contract only when request is Approved/Deposited and payment is successful, then update room/status accordingly.</t>
+  </si>
+  <si>
+    <t>Contract creation backend flow</t>
+  </si>
+  <si>
+    <t>Checking only that the user role is Landlord is enough for room/request APIs.</t>
+  </si>
+  <si>
+    <t>A landlord must also own the room/request resource; otherwise one landlord may modify another landlord's data.</t>
+  </si>
+  <si>
+    <t>Reviewed API authorization logic and User → Room relationship in the database.</t>
+  </si>
+  <si>
+    <t>Add ownership checks using landlordId in update/delete/approve/reject queries.</t>
+  </si>
+  <si>
+    <t>A room only needs Available/Unavailable status after contract creation.</t>
+  </si>
+  <si>
+    <t>RentalRoom needs clearer statuses such as Available, Pending Deposit, Rented, Hidden/Inactive to handle approval, deposit, and contract flow.</t>
+  </si>
+  <si>
+    <t>Compared rental request lifecycle with room listing visibility and contract creation flow.</t>
+  </si>
+  <si>
+    <t>Update room/request status only after successful deposit and contract creation; keep listing states separated.</t>
+  </si>
+  <si>
+    <t>Có – tách landlord backend thành room/request/contract/dashboard để team dễ code</t>
+  </si>
+  <si>
+    <t>Có – validation Room API giúp tránh dữ liệu phòng thiếu giá, diện tích, địa chỉ, tiện ích</t>
+  </si>
+  <si>
+    <t>Có – approval flow đúng logic landlord duyệt trước rồi tenant mới cọc</t>
+  </si>
+  <si>
+    <t>Có – kiểm tra ownership giúp landlord không sửa phòng/yêu cầu của người khác</t>
+  </si>
+  <si>
+    <t>Có – contract chỉ tạo sau khi request/deposit hợp lệ để tránh sai nghiệp vụ</t>
   </si>
 </sst>
 </file>
@@ -1079,18 +1193,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1153,27 +1261,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1185,13 +1290,13 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1215,6 +1320,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1231,14 +1345,23 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1553,14 +1676,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
     </row>
     <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -1608,24 +1731,24 @@
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="16">
-        <v>140</v>
+      <c r="C10" s="15">
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="17">
-        <v>25</v>
+      <c r="C11" s="16">
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="18">
-        <v>0.17860000000000001</v>
+      <c r="C12" s="17">
+        <v>0.17649999999999999</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>10</v>
@@ -1635,8 +1758,8 @@
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="17">
-        <v>8</v>
+      <c r="C13" s="16">
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" x14ac:dyDescent="0.35">
@@ -1662,7 +1785,7 @@
       <c r="A17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="18" t="s">
         <v>106</v>
       </c>
       <c r="C17" s="5" t="s">
@@ -1673,30 +1796,30 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="18" t="s">
         <v>108</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="18" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="19" t="s">
+      <c r="D19" s="18" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1704,27 +1827,27 @@
       <c r="A20" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="C20" s="19" t="s">
+      <c r="C20" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D20" s="19" t="s">
+      <c r="D20" s="18" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="15" t="s">
         <v>119</v>
       </c>
     </row>
@@ -1733,7 +1856,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>22</v>
       </c>
@@ -1744,47 +1867,47 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="6">
-        <v>5</v>
-      </c>
-      <c r="C24" s="7" t="s">
+      <c r="B24" s="33">
+        <v>6</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="6">
-        <v>6</v>
-      </c>
-      <c r="C25" s="7" t="s">
+      <c r="B25" s="33">
+        <v>7</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="6">
-        <v>7</v>
-      </c>
-      <c r="C26" s="7" t="s">
+      <c r="B26" s="33">
+        <v>8</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="6">
-        <v>7</v>
-      </c>
-      <c r="C27" s="7" t="s">
+      <c r="B27" s="33">
+        <v>9</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1798,7 +1921,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1810,31 +1933,31 @@
     <col min="8" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-    </row>
-    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+    </row>
+    <row r="2" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-    </row>
-    <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+    </row>
+    <row r="3" spans="1:10" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>32</v>
       </c>
@@ -1860,655 +1983,841 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="100.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="5">
+    <row r="4" spans="1:10" ht="100.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="37">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="37" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="35" t="s">
         <v>160</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="35" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="100.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="5">
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+    </row>
+    <row r="5" spans="1:10" ht="100.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="37">
         <v>2</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="35" t="s">
         <v>124</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="35" t="s">
         <v>161</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="35" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="100.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="5">
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+    </row>
+    <row r="6" spans="1:10" ht="100.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="37">
         <v>3</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="35" t="s">
         <v>152</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="35" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="106.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="5">
+      <c r="I6" s="36"/>
+      <c r="J6" s="36"/>
+    </row>
+    <row r="7" spans="1:10" ht="106.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="37">
         <v>4</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="35" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="104.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="5">
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
+    </row>
+    <row r="8" spans="1:10" ht="104.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="37">
         <v>5</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="35" t="s">
         <v>154</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="35" t="s">
         <v>132</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="35" t="s">
         <v>133</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="35" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="137.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="5">
+      <c r="I8" s="36"/>
+      <c r="J8" s="36"/>
+    </row>
+    <row r="9" spans="1:10" ht="137.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="37">
         <v>6</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="35" t="s">
         <v>155</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="35" t="s">
         <v>134</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="35" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="108.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="5">
+      <c r="I9" s="36"/>
+      <c r="J9" s="36"/>
+    </row>
+    <row r="10" spans="1:10" ht="108.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="37">
         <v>7</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="35" t="s">
         <v>156</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="35" t="s">
         <v>138</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="35" t="s">
         <v>166</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="H10" s="35" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="89.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="5">
+      <c r="I10" s="36"/>
+      <c r="J10" s="36"/>
+    </row>
+    <row r="11" spans="1:10" ht="89.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="37">
         <v>8</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="35" t="s">
         <v>157</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="35" t="s">
         <v>141</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="35" t="s">
         <v>142</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="35" t="s">
         <v>167</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="H11" s="35" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="103.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="5">
+      <c r="I11" s="36"/>
+      <c r="J11" s="36"/>
+    </row>
+    <row r="12" spans="1:10" ht="103.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="37">
         <v>9</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="35" t="s">
         <v>158</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="35" t="s">
         <v>168</v>
       </c>
-      <c r="H12" s="19" t="s">
+      <c r="H12" s="35" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="118.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="5">
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
+    </row>
+    <row r="13" spans="1:10" ht="118.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="37">
         <v>10</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="35" t="s">
         <v>159</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="H13" s="19" t="s">
+      <c r="H13" s="35" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="19">
+      <c r="I13" s="36"/>
+      <c r="J13" s="36"/>
+    </row>
+    <row r="14" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="35">
         <v>11</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="35" t="s">
         <v>197</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="35" t="s">
         <v>198</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="35" t="s">
         <v>199</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="35" t="s">
         <v>200</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="35" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="5">
+      <c r="I14" s="36"/>
+      <c r="J14" s="36"/>
+    </row>
+    <row r="15" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="37">
         <v>12</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="35" t="s">
         <v>202</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="35" t="s">
         <v>203</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="35" t="s">
         <v>204</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="35" t="s">
         <v>205</v>
       </c>
-      <c r="H15" s="19" t="s">
+      <c r="H15" s="35" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="5">
+      <c r="I15" s="36"/>
+      <c r="J15" s="36"/>
+    </row>
+    <row r="16" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="37">
         <v>13</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="35" t="s">
         <v>209</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="35" t="s">
         <v>210</v>
       </c>
-      <c r="H16" s="19" t="s">
+      <c r="H16" s="35" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="5">
+      <c r="I16" s="36"/>
+      <c r="J16" s="36"/>
+    </row>
+    <row r="17" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="37">
         <v>14</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="37" t="s">
         <v>212</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="E17" s="35" t="s">
         <v>213</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="F17" s="35" t="s">
         <v>214</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="35" t="s">
         <v>215</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="H17" s="35" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="5">
+      <c r="I17" s="36"/>
+      <c r="J17" s="36"/>
+    </row>
+    <row r="18" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="37">
         <v>15</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="35" t="s">
         <v>217</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="E18" s="35" t="s">
         <v>218</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="F18" s="35" t="s">
         <v>219</v>
       </c>
-      <c r="G18" s="19" t="s">
+      <c r="G18" s="35" t="s">
         <v>220</v>
       </c>
-      <c r="H18" s="19" t="s">
+      <c r="H18" s="35" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="19">
+      <c r="I18" s="36"/>
+      <c r="J18" s="36"/>
+    </row>
+    <row r="19" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="35">
         <v>16</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="19" t="s">
+      <c r="D19" s="35" t="s">
         <v>242</v>
       </c>
-      <c r="E19" s="19" t="s">
+      <c r="E19" s="35" t="s">
         <v>243</v>
       </c>
-      <c r="F19" s="19" t="s">
+      <c r="F19" s="35" t="s">
         <v>244</v>
       </c>
-      <c r="G19" s="19" t="s">
+      <c r="G19" s="35" t="s">
         <v>245</v>
       </c>
-      <c r="H19" s="19" t="s">
+      <c r="H19" s="35" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="19">
+      <c r="I19" s="36"/>
+      <c r="J19" s="36"/>
+    </row>
+    <row r="20" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="35">
         <v>17</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="19" t="s">
+      <c r="C20" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="19" t="s">
+      <c r="D20" s="35" t="s">
         <v>247</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="E20" s="35" t="s">
         <v>248</v>
       </c>
-      <c r="F20" s="19" t="s">
+      <c r="F20" s="35" t="s">
         <v>249</v>
       </c>
-      <c r="G20" s="19" t="s">
+      <c r="G20" s="35" t="s">
         <v>250</v>
       </c>
-      <c r="H20" s="19" t="s">
+      <c r="H20" s="35" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="19">
+      <c r="I20" s="36"/>
+      <c r="J20" s="36"/>
+    </row>
+    <row r="21" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="35">
         <v>18</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="19" t="s">
+      <c r="C21" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="19" t="s">
+      <c r="D21" s="35" t="s">
         <v>252</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="E21" s="35" t="s">
         <v>253</v>
       </c>
-      <c r="F21" s="19" t="s">
+      <c r="F21" s="35" t="s">
         <v>254</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="35" t="s">
         <v>255</v>
       </c>
-      <c r="H21" s="19" t="s">
+      <c r="H21" s="35" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="19">
+      <c r="I21" s="36"/>
+      <c r="J21" s="36"/>
+    </row>
+    <row r="22" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="35">
         <v>19</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C22" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="19" t="s">
+      <c r="D22" s="35" t="s">
         <v>257</v>
       </c>
-      <c r="E22" s="19" t="s">
+      <c r="E22" s="35" t="s">
         <v>258</v>
       </c>
-      <c r="F22" s="19" t="s">
+      <c r="F22" s="35" t="s">
         <v>259</v>
       </c>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="35" t="s">
         <v>260</v>
       </c>
-      <c r="H22" s="19" t="s">
+      <c r="H22" s="35" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="19">
+      <c r="I22" s="36"/>
+      <c r="J22" s="36"/>
+    </row>
+    <row r="23" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="35">
         <v>20</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="35" t="s">
         <v>262</v>
       </c>
-      <c r="E23" s="19" t="s">
+      <c r="E23" s="35" t="s">
         <v>263</v>
       </c>
-      <c r="F23" s="19" t="s">
+      <c r="F23" s="35" t="s">
         <v>264</v>
       </c>
-      <c r="G23" s="19" t="s">
+      <c r="G23" s="35" t="s">
         <v>265</v>
       </c>
-      <c r="H23" s="19" t="s">
+      <c r="H23" s="35" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="19">
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
+    </row>
+    <row r="24" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="35">
         <v>21</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="19" t="s">
+      <c r="C24" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="19" t="s">
+      <c r="D24" s="35" t="s">
         <v>267</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E24" s="35" t="s">
         <v>268</v>
       </c>
-      <c r="F24" s="19" t="s">
+      <c r="F24" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="G24" s="19" t="s">
+      <c r="G24" s="35" t="s">
         <v>270</v>
       </c>
-      <c r="H24" s="19" t="s">
+      <c r="H24" s="35" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="19">
+      <c r="I24" s="36"/>
+      <c r="J24" s="36"/>
+    </row>
+    <row r="25" spans="1:10" ht="79.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="35">
         <v>22</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="C25" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="19" t="s">
+      <c r="D25" s="35" t="s">
         <v>272</v>
       </c>
-      <c r="E25" s="19" t="s">
+      <c r="E25" s="35" t="s">
         <v>273</v>
       </c>
-      <c r="F25" s="19" t="s">
+      <c r="F25" s="35" t="s">
         <v>274</v>
       </c>
-      <c r="G25" s="19" t="s">
+      <c r="G25" s="35" t="s">
         <v>275</v>
       </c>
-      <c r="H25" s="19" t="s">
+      <c r="H25" s="35" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" ht="123.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="19">
+      <c r="I25" s="36"/>
+      <c r="J25" s="36"/>
+    </row>
+    <row r="26" spans="1:10" ht="123.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="35">
         <v>23</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="C26" s="19" t="s">
+      <c r="C26" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="19" t="s">
+      <c r="D26" s="35" t="s">
         <v>277</v>
       </c>
-      <c r="E26" s="19" t="s">
+      <c r="E26" s="35" t="s">
         <v>278</v>
       </c>
-      <c r="F26" s="19" t="s">
+      <c r="F26" s="35" t="s">
         <v>279</v>
       </c>
-      <c r="G26" s="19" t="s">
+      <c r="G26" s="35" t="s">
         <v>280</v>
       </c>
-      <c r="H26" s="19" t="s">
+      <c r="H26" s="35" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="31">
+      <c r="I26" s="36"/>
+      <c r="J26" s="36"/>
+    </row>
+    <row r="27" spans="1:10" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="38">
         <v>24</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="31" t="s">
+      <c r="C27" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="31" t="s">
+      <c r="D27" s="38" t="s">
         <v>282</v>
       </c>
-      <c r="E27" s="31" t="s">
+      <c r="E27" s="38" t="s">
         <v>283</v>
       </c>
-      <c r="F27" s="31" t="s">
+      <c r="F27" s="38" t="s">
         <v>284</v>
       </c>
-      <c r="G27" s="31" t="s">
+      <c r="G27" s="38" t="s">
         <v>285</v>
       </c>
-      <c r="H27" s="31" t="s">
+      <c r="H27" s="38" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" ht="66" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="31">
+      <c r="I27" s="36"/>
+      <c r="J27" s="36"/>
+    </row>
+    <row r="28" spans="1:10" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="38">
         <v>25</v>
       </c>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="31" t="s">
+      <c r="C28" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="D28" s="31" t="s">
+      <c r="D28" s="38" t="s">
         <v>287</v>
       </c>
-      <c r="E28" s="31" t="s">
+      <c r="E28" s="38" t="s">
         <v>288</v>
       </c>
-      <c r="F28" s="31" t="s">
+      <c r="F28" s="38" t="s">
         <v>289</v>
       </c>
-      <c r="G28" s="31" t="s">
+      <c r="G28" s="38" t="s">
         <v>290</v>
       </c>
-      <c r="H28" s="31" t="s">
+      <c r="H28" s="38" t="s">
         <v>291</v>
       </c>
+      <c r="I28" s="36"/>
+      <c r="J28" s="36"/>
+    </row>
+    <row r="29" spans="1:10" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="34">
+        <v>26</v>
+      </c>
+      <c r="B29" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="C29" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="35" t="s">
+        <v>314</v>
+      </c>
+      <c r="E29" s="35" t="s">
+        <v>315</v>
+      </c>
+      <c r="F29" s="35" t="s">
+        <v>316</v>
+      </c>
+      <c r="G29" s="35" t="s">
+        <v>317</v>
+      </c>
+      <c r="H29" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="I29" s="36"/>
+      <c r="J29" s="36"/>
+    </row>
+    <row r="30" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="36">
+        <v>27</v>
+      </c>
+      <c r="B30" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="D30" s="38" t="s">
+        <v>319</v>
+      </c>
+      <c r="E30" s="38" t="s">
+        <v>320</v>
+      </c>
+      <c r="F30" s="38" t="s">
+        <v>321</v>
+      </c>
+      <c r="G30" s="38" t="s">
+        <v>322</v>
+      </c>
+      <c r="H30" s="38" t="s">
+        <v>323</v>
+      </c>
+      <c r="I30" s="36"/>
+    </row>
+    <row r="31" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A31" s="36">
+        <v>28</v>
+      </c>
+      <c r="B31" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="D31" s="38" t="s">
+        <v>324</v>
+      </c>
+      <c r="E31" s="38" t="s">
+        <v>325</v>
+      </c>
+      <c r="F31" s="38" t="s">
+        <v>326</v>
+      </c>
+      <c r="G31" s="38" t="s">
+        <v>327</v>
+      </c>
+      <c r="H31" s="38" t="s">
+        <v>328</v>
+      </c>
+      <c r="I31" s="36"/>
+    </row>
+    <row r="32" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="36">
+        <v>29</v>
+      </c>
+      <c r="B32" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="38" t="s">
+        <v>28</v>
+      </c>
+      <c r="D32" s="38" t="s">
+        <v>329</v>
+      </c>
+      <c r="E32" s="38" t="s">
+        <v>330</v>
+      </c>
+      <c r="F32" s="38" t="s">
+        <v>331</v>
+      </c>
+      <c r="G32" s="38" t="s">
+        <v>333</v>
+      </c>
+      <c r="H32" s="38" t="s">
+        <v>332</v>
+      </c>
+      <c r="I32" s="36"/>
+    </row>
+    <row r="33" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="36">
+        <v>30</v>
+      </c>
+      <c r="B33" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="D33" s="38" t="s">
+        <v>334</v>
+      </c>
+      <c r="E33" s="38" t="s">
+        <v>335</v>
+      </c>
+      <c r="F33" s="38" t="s">
+        <v>336</v>
+      </c>
+      <c r="G33" s="38" t="s">
+        <v>337</v>
+      </c>
+      <c r="H33" s="38" t="s">
+        <v>338</v>
+      </c>
+      <c r="I33" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2530,24 +2839,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
     </row>
     <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
@@ -2573,19 +2882,19 @@
       <c r="A4" s="5">
         <v>2</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>173</v>
       </c>
     </row>
@@ -2593,19 +2902,19 @@
       <c r="A5" s="5">
         <v>6</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>176</v>
       </c>
     </row>
@@ -2613,19 +2922,19 @@
       <c r="A6" s="5">
         <v>10</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>181</v>
       </c>
     </row>
@@ -2633,19 +2942,19 @@
       <c r="A7" s="5">
         <v>11</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>222</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>228</v>
       </c>
     </row>
@@ -2653,97 +2962,121 @@
       <c r="A8" s="5">
         <v>14</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>227</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="19">
+      <c r="A9" s="18">
         <v>19</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>292</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>295</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>298</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="19">
+      <c r="A10" s="18">
         <v>23</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>293</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>296</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>299</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="19">
+      <c r="A11" s="18">
         <v>24</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>294</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>297</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-    </row>
-    <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
+    <row r="12" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="18">
+        <v>29</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>339</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="5">
+        <v>30</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>343</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>346</v>
+      </c>
     </row>
     <row r="14" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
@@ -2839,13 +3172,13 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="7" t="s">
         <v>55</v>
       </c>
     </row>
@@ -2915,7 +3248,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2925,20 +3258,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
     </row>
     <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -2949,83 +3282,83 @@
       <c r="A5" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>74</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="8" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>182</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="21" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="21" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="21" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="22" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="21" t="s">
         <v>187</v>
       </c>
     </row>
@@ -3038,98 +3371,98 @@
       <c r="A13" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>74</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="21" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="D15" s="22" t="s">
+      <c r="D15" s="21" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="21" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="D17" s="22" t="s">
+      <c r="D17" s="21" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="21" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="11" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="12" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="12" t="s">
         <v>96</v>
       </c>
     </row>
@@ -3139,26 +3472,26 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="13" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A27" s="15" t="s">
+      <c r="A27" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="7">
+      <c r="A28" s="6">
         <v>1</v>
       </c>
       <c r="B28" t="s">
@@ -3172,7 +3505,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="7">
+      <c r="A29" s="6">
         <v>2</v>
       </c>
       <c r="B29" t="s">
@@ -3186,7 +3519,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="7">
+      <c r="A30" s="6">
         <v>3</v>
       </c>
       <c r="B30" t="s">
@@ -3200,10 +3533,10 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="24">
+      <c r="A31" s="23">
         <v>4</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="15" t="s">
         <v>230</v>
       </c>
       <c r="C31" t="s">
@@ -3214,10 +3547,10 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="24">
+      <c r="A32" s="23">
         <v>5</v>
       </c>
-      <c r="B32" s="16" t="s">
+      <c r="B32" s="15" t="s">
         <v>231</v>
       </c>
       <c r="C32" t="s">
@@ -3228,10 +3561,10 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="24">
+      <c r="A33" s="23">
         <v>6</v>
       </c>
-      <c r="B33" s="16" t="s">
+      <c r="B33" s="15" t="s">
         <v>232</v>
       </c>
       <c r="C33" t="s">
@@ -3242,10 +3575,10 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="24">
+      <c r="A34" s="23">
         <v>7</v>
       </c>
-      <c r="B34" s="16" t="s">
+      <c r="B34" s="15" t="s">
         <v>233</v>
       </c>
       <c r="C34" t="s">
@@ -3256,10 +3589,10 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="24">
+      <c r="A35" s="23">
         <v>8</v>
       </c>
-      <c r="B35" s="16" t="s">
+      <c r="B35" s="15" t="s">
         <v>234</v>
       </c>
       <c r="C35" t="s">
@@ -3270,10 +3603,10 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="24">
+      <c r="A36" s="23">
         <v>9</v>
       </c>
-      <c r="B36" s="16" t="s">
+      <c r="B36" s="15" t="s">
         <v>235</v>
       </c>
       <c r="C36" t="s">
@@ -3284,10 +3617,10 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="24">
+      <c r="A37" s="23">
         <v>10</v>
       </c>
-      <c r="B37" s="16" t="s">
+      <c r="B37" s="15" t="s">
         <v>236</v>
       </c>
       <c r="C37" t="s">
@@ -3298,10 +3631,10 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="24">
+      <c r="A38" s="23">
         <v>11</v>
       </c>
-      <c r="B38" s="16" t="s">
+      <c r="B38" s="15" t="s">
         <v>237</v>
       </c>
       <c r="C38" t="s">
@@ -3312,10 +3645,10 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="24">
+      <c r="A39" s="23">
         <v>12</v>
       </c>
-      <c r="B39" s="16" t="s">
+      <c r="B39" s="15" t="s">
         <v>238</v>
       </c>
       <c r="C39" t="s">
@@ -3326,10 +3659,10 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="24">
+      <c r="A40" s="23">
         <v>13</v>
       </c>
-      <c r="B40" s="16" t="s">
+      <c r="B40" s="15" t="s">
         <v>239</v>
       </c>
       <c r="C40" t="s">
@@ -3340,10 +3673,10 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="24">
+      <c r="A41" s="23">
         <v>14</v>
       </c>
-      <c r="B41" s="16" t="s">
+      <c r="B41" s="15" t="s">
         <v>240</v>
       </c>
       <c r="C41" t="s">
@@ -3354,10 +3687,10 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="24">
+      <c r="A42" s="23">
         <v>15</v>
       </c>
-      <c r="B42" s="16" t="s">
+      <c r="B42" s="15" t="s">
         <v>241</v>
       </c>
       <c r="C42" t="s">
@@ -3368,10 +3701,10 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A43" s="32">
+      <c r="A43" s="25">
         <v>16</v>
       </c>
-      <c r="B43" s="31" t="s">
+      <c r="B43" s="24" t="s">
         <v>304</v>
       </c>
       <c r="C43" t="s">
@@ -3382,10 +3715,10 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="33">
+      <c r="A44" s="26">
         <v>17</v>
       </c>
-      <c r="B44" s="31" t="s">
+      <c r="B44" s="24" t="s">
         <v>305</v>
       </c>
       <c r="C44" t="s">
@@ -3396,10 +3729,10 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45" s="24">
+      <c r="A45" s="23">
         <v>18</v>
       </c>
-      <c r="B45" s="31" t="s">
+      <c r="B45" s="24" t="s">
         <v>306</v>
       </c>
       <c r="C45" t="s">
@@ -3410,10 +3743,10 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" s="24">
+      <c r="A46" s="23">
         <v>19</v>
       </c>
-      <c r="B46" s="31" t="s">
+      <c r="B46" s="24" t="s">
         <v>307</v>
       </c>
       <c r="C46" t="s">
@@ -3424,10 +3757,10 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="24">
+      <c r="A47" s="23">
         <v>20</v>
       </c>
-      <c r="B47" s="31" t="s">
+      <c r="B47" s="24" t="s">
         <v>308</v>
       </c>
       <c r="C47" t="s">
@@ -3438,10 +3771,10 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" s="24">
+      <c r="A48" s="23">
         <v>21</v>
       </c>
-      <c r="B48" s="31" t="s">
+      <c r="B48" s="24" t="s">
         <v>309</v>
       </c>
       <c r="C48" t="s">
@@ -3452,10 +3785,10 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="24">
+      <c r="A49" s="23">
         <v>22</v>
       </c>
-      <c r="B49" s="31" t="s">
+      <c r="B49" s="24" t="s">
         <v>310</v>
       </c>
       <c r="C49" t="s">
@@ -3466,10 +3799,10 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" s="24">
+      <c r="A50" s="23">
         <v>23</v>
       </c>
-      <c r="B50" s="31" t="s">
+      <c r="B50" s="24" t="s">
         <v>311</v>
       </c>
       <c r="C50" t="s">
@@ -3480,10 +3813,10 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="24">
+      <c r="A51" s="23">
         <v>24</v>
       </c>
-      <c r="B51" s="31" t="s">
+      <c r="B51" s="24" t="s">
         <v>312</v>
       </c>
       <c r="C51" t="s">
@@ -3494,16 +3827,86 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A52" s="24">
+      <c r="A52" s="23">
         <v>25</v>
       </c>
-      <c r="B52" s="31" t="s">
+      <c r="B52" s="24" t="s">
         <v>313</v>
       </c>
       <c r="C52" t="s">
         <v>196</v>
       </c>
       <c r="D52" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A53" s="23">
+        <v>26</v>
+      </c>
+      <c r="B53" s="15" t="s">
+        <v>347</v>
+      </c>
+      <c r="C53" t="s">
+        <v>196</v>
+      </c>
+      <c r="D53" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A54" s="23">
+        <v>27</v>
+      </c>
+      <c r="B54" s="15" t="s">
+        <v>348</v>
+      </c>
+      <c r="C54" t="s">
+        <v>196</v>
+      </c>
+      <c r="D54" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="23">
+        <v>28</v>
+      </c>
+      <c r="B55" s="15" t="s">
+        <v>349</v>
+      </c>
+      <c r="C55" t="s">
+        <v>196</v>
+      </c>
+      <c r="D55" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A56" s="23">
+        <v>29</v>
+      </c>
+      <c r="B56" s="15" t="s">
+        <v>350</v>
+      </c>
+      <c r="C56" t="s">
+        <v>196</v>
+      </c>
+      <c r="D56" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" s="23">
+        <v>30</v>
+      </c>
+      <c r="B57" s="15" t="s">
+        <v>351</v>
+      </c>
+      <c r="C57" t="s">
+        <v>196</v>
+      </c>
+      <c r="D57" t="s">
         <v>196</v>
       </c>
     </row>

</xml_diff>